<commit_message>
Modified 6 materials to be consistent with 3 materials
</commit_message>
<xml_diff>
--- a/DataVaryingTemperature/6MaterialsTempDependent.xlsx
+++ b/DataVaryingTemperature/6MaterialsTempDependent.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\DataVaryingTemperature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E348C81-E2A9-4428-9731-3413BB4A78DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE421A2-E897-4D9A-9AEC-8B1B89B1C30F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="228" yWindow="1740" windowWidth="20604" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -653,34 +653,34 @@
         <v>14</v>
       </c>
       <c r="B3" s="4">
-        <v>8000</v>
+        <v>7850</v>
       </c>
       <c r="C3" s="4">
         <v>6</v>
       </c>
       <c r="D3" s="6">
-        <v>200000000000</v>
+        <v>210000000000</v>
       </c>
       <c r="E3" s="6">
-        <v>120000000000</v>
+        <v>12000000000</v>
       </c>
       <c r="F3" s="6">
-        <v>90000000000</v>
+        <v>9000000000</v>
       </c>
       <c r="G3" s="6">
-        <v>80000000000</v>
+        <v>800000000</v>
       </c>
       <c r="H3" s="6">
-        <v>900000000</v>
+        <v>250000000</v>
       </c>
       <c r="I3" s="6">
-        <v>800000000</v>
+        <v>80000000</v>
       </c>
       <c r="J3" s="6">
-        <v>700000000</v>
+        <v>7000000</v>
       </c>
       <c r="K3" s="6">
-        <v>650000000</v>
+        <v>650000</v>
       </c>
       <c r="L3" s="6">
         <v>18</v>
@@ -712,28 +712,28 @@
         <v>4</v>
       </c>
       <c r="D4" s="6">
-        <v>190000000000</v>
+        <v>200000000000</v>
       </c>
       <c r="E4" s="6">
-        <v>110000000000</v>
+        <v>11000000000</v>
       </c>
       <c r="F4" s="6">
-        <v>90000000000</v>
+        <v>9000000000</v>
       </c>
       <c r="G4" s="6">
-        <v>80000000000</v>
+        <v>800000000</v>
       </c>
       <c r="H4" s="6">
-        <v>700000000</v>
+        <v>180000000</v>
       </c>
       <c r="I4" s="6">
-        <v>600000000</v>
+        <v>60000000</v>
       </c>
       <c r="J4" s="6">
-        <v>550000000</v>
+        <v>5500000</v>
       </c>
       <c r="K4" s="6">
-        <v>500000000</v>
+        <v>500000</v>
       </c>
       <c r="L4" s="6">
         <v>50</v>
@@ -759,16 +759,16 @@
         <v>15</v>
       </c>
       <c r="B5" s="4">
-        <v>2800</v>
+        <v>2700</v>
       </c>
       <c r="C5" s="4">
         <v>2</v>
       </c>
       <c r="D5" s="6">
-        <v>73000000000</v>
+        <v>70000000000</v>
       </c>
       <c r="E5" s="6">
-        <v>40000000000</v>
+        <v>4000000000</v>
       </c>
       <c r="F5" s="6">
         <v>20000000</v>
@@ -777,16 +777,16 @@
         <v>2000000</v>
       </c>
       <c r="H5" s="6">
-        <v>300000000</v>
+        <v>100000000</v>
       </c>
       <c r="I5" s="6">
-        <v>100000000</v>
+        <v>1000000</v>
       </c>
       <c r="J5" s="6">
-        <v>2000000</v>
+        <v>200000</v>
       </c>
       <c r="K5" s="6">
-        <v>100000</v>
+        <v>10000</v>
       </c>
       <c r="L5" s="6">
         <v>190</v>
@@ -874,22 +874,22 @@
         <v>200000000000</v>
       </c>
       <c r="E7" s="6">
-        <v>190000000000</v>
+        <v>3000000000</v>
       </c>
       <c r="F7" s="6">
-        <v>160000000000</v>
+        <v>160000000</v>
       </c>
       <c r="G7" s="6">
         <v>10000000</v>
       </c>
       <c r="H7" s="6">
-        <v>860000000</v>
+        <v>86000000</v>
       </c>
       <c r="I7" s="6">
-        <v>700000000</v>
+        <v>40000000</v>
       </c>
       <c r="J7" s="6">
-        <v>450000000</v>
+        <v>4500000</v>
       </c>
       <c r="K7" s="6">
         <v>600000</v>

</xml_diff>